<commit_message>
Add indoor GIS files and resources for Week 08 and Week 09
- Created XML message files for indoor GIS operations.
- Added import log XML file for tracking imports.
- Included various thumbnail images for indoor GIS indexing.
- Added multiple binary files related to indoor GIS indexing and data storage.
- Introduced ArcGIS project files (.aprx, .atbx) and geodatabase files (.gdb) for indoor GIS.
- Updated RMSE data files for Weeks 08 and 09.
- Added PowerPoint presentation for accuracy lecture in Week 09.
</commit_message>
<xml_diff>
--- a/docs/Lectures/Week08/rmse_data.xlsx
+++ b/docs/Lectures/Week08/rmse_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UCA\classes\2021Fall\GIS3403 1800\Lectures\data\Lecture6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ConwayTeaching\GIS_I\GIS_I\docs\Lectures\Week08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB02972-E62F-4636-88A7-E99BCE374635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F06D13-601B-4642-9DE6-04B77CE3AAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -75,11 +75,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -88,6 +88,13 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -172,7 +179,7 @@
     <xf numFmtId="4" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -457,19 +464,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="26.375" customWidth="1"/>
+    <col min="3" max="3" width="21.375" customWidth="1"/>
+    <col min="4" max="4" width="25.625" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="6" max="6" width="15.625" customWidth="1"/>
+    <col min="7" max="7" width="11.625" customWidth="1"/>
+    <col min="8" max="8" width="15.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -495,7 +502,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="16.5" thickBot="1">
       <c r="A2" s="3">
         <v>513128.4</v>
       </c>
@@ -512,7 +519,7 @@
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="16.5" thickBot="1">
       <c r="A3" s="3">
         <v>513117.8</v>
       </c>
@@ -529,7 +536,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="16.5" thickBot="1">
       <c r="A4" s="3">
         <v>513201.7</v>
       </c>
@@ -546,7 +553,7 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
     </row>
-    <row r="5" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="16.5" thickBot="1">
       <c r="A5" s="3">
         <v>513180.3</v>
       </c>
@@ -563,7 +570,7 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="16.5" thickBot="1">
       <c r="A6" s="3">
         <v>513215.6</v>
       </c>
@@ -580,13 +587,13 @@
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="E7" t="s">
         <v>6</v>
       </c>
       <c r="F7" s="6"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="E8" t="s">
         <v>3</v>
       </c>
@@ -595,12 +602,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="E9" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>